<commit_message>
Catalog update — Rob — 2026-08-26 17:10 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,7 +9,8 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Alt Codes" sheetId="2" r:id="rId6"/>
+    <sheet name="Discontinued" sheetId="3" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -48159,153 +48160,296 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="42"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="28" t="s">
-        <v>4390</v>
-      </c>
-      <c r="B1" s="28" t="s">
-        <v>4391</v>
-      </c>
-      <c r="C1" s="28" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="28" t="s">
-        <v>4392</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>4393</v>
-      </c>
-      <c r="B2" s="0" t="s">
-        <v>4394</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>463</v>
-      </c>
-      <c r="D2" s="0" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>4393</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>4395</v>
-      </c>
-      <c r="C3" s="0" t="s">
-        <v>1218</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>1219</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>4393</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>4396</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>1223</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>1224</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>4393</v>
-      </c>
-      <c r="B5" s="0" t="s">
-        <v>4397</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>1226</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>1227</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>4398</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>4399</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>503</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>4400</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>4401</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>2427</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>2428</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>4400</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>4402</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>4403</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>4400</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>4404</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>4405</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>30</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer Code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peats Code</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHERAX55</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHER AX55</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Wi-Fi 6 Router AX3000 Dual-Band Wi-Fi 6 Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVR2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVR2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVRS2SD128GBU3</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD128GBU3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rob-test</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BLK</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BK</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groove  Black Portable CD Player</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100H</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOH100</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FB1001100EUS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC2250100EUS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4250P100EUS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4260P100EUS</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4360B100EUS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B6"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-26 17:55 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,8 +9,8 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="2" r:id="rId6"/>
-    <sheet name="Discontinued" sheetId="3" r:id="rId7"/>
+    <sheet name="Alt Codes" sheetId="4" r:id="rId8"/>
+    <sheet name="Discontinued" sheetId="5" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -48404,7 +48404,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC2250100EUS</t>
+          <t xml:space="preserve">ICFP27.CE7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -48416,7 +48416,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4250P100EUS</t>
+          <t xml:space="preserve">ICFP37.CE7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -48428,7 +48428,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4260P100EUS</t>
+          <t xml:space="preserve">SRS-NS7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -48440,7 +48440,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4360B100EUS</t>
+          <t xml:space="preserve">VMC2250100EUS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -48449,7 +48449,43 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4250P100EUS</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4260P100EUS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4360B100EUS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:B9"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-26 18:25 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,8 +9,8 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="4" r:id="rId8"/>
-    <sheet name="Discontinued" sheetId="5" r:id="rId9"/>
+    <sheet name="Alt Codes" sheetId="6" r:id="rId10"/>
+    <sheet name="Discontinued" sheetId="7" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -48192,181 +48192,775 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHER MR200</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MR200</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LTE/5G Gateway AC750 Wireless Dual Band 4G LTE Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHERC50V3</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHER C50V3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Router AC1200 Dual Band Wireless Cable Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4KIT</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4 KIT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVPSR760HB.CEK</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVPSR760HBCEK</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony DVD player with Picture enhcancing technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSD40.CEK</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSD40CEK</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony 2.1chl Soundbar with powerful Wireless Subwoofer inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSF150.CEK</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSF150CEK</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony 2chl Single Soundbar with Bluetooth</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICF506.CEK</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICF506CEK</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony portable AM/FM radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1B.CEK</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1BCEK</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black AM/FM clock radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1W.CEK</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1WCEK</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White AM/FM clock radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAXMINIFILM</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10B.CE7</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10BCE7</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black Portable BT Speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10W.CE7</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10WCE7</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White Portable BT Speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100B.CE7</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100BCE7</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black Waterproof BT Speaker, EXTRA BASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100D.CE7</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100DCE7</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Orange Compact BT Wirelss Spkr</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100H.CE7</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100HCE7</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Light Grey Waterproof BT Speaker, EXTRA BASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100L.CE7</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100LCE7</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Light Blue Waterproof BT Speaker, EXTRA BASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC100</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC200</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC310</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C310</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO P100</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA8631PKIT</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA8631P KIT</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link AV1300/AV2000 Powerline Adapter AV1300 Gigabit</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t xml:space="preserve">ARCHERAX55</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t xml:space="preserve">ARCHER AX55</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Wi-Fi 6 Router AX3000 Dual-Band Wi-Fi 6 Router</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="30">
+      <c r="A30" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t xml:space="preserve">DVR2SD32GBU3</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="31">
+      <c r="A31" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t xml:space="preserve">DVR2SD64GBU3</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD64GBU3</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t xml:space="preserve">DVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t xml:space="preserve">rob-test</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t xml:space="preserve">WPA7517KITV2</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t xml:space="preserve">WPA7517KIT V2</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t xml:space="preserve">soundstore</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t xml:space="preserve">GVPS110BLK</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t xml:space="preserve">GVPS110BK</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t xml:space="preserve">Groove  Black Portable CD Player</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t xml:space="preserve">soundstore</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOL510E</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPO L510E</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t xml:space="preserve">soundstore</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOP100H</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOH100</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D36"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Catalog update — Al — 2026-08-27 14:21 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,8 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="6" r:id="rId10"/>
-    <sheet name="Discontinued" sheetId="7" r:id="rId11"/>
+    <sheet name="Alt Codes" sheetId="8" r:id="rId12"/>
+    <sheet name="Discontinued" sheetId="9" r:id="rId13"/>
+    <sheet name="Legit Codes" sheetId="10" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -49082,4 +49083,40 @@
   </sheetData>
   <autoFilter ref="A1:B9"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="44" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOD235</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-27 16:10 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="8" r:id="rId12"/>
-    <sheet name="Discontinued" sheetId="9" r:id="rId13"/>
-    <sheet name="Legit Codes" sheetId="10" r:id="rId14"/>
+    <sheet name="Alt Codes" sheetId="11" r:id="rId15"/>
+    <sheet name="Discontinued" sheetId="12" r:id="rId16"/>
+    <sheet name="Legit Codes" sheetId="13" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -49107,7 +49107,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOD235</t>
+          <t xml:space="preserve">100315</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -49116,7 +49116,67 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVBT1200BK</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HAS36WA</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1023R</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX310APBCE7</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS816</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B2"/>
+  <autoFilter ref="A1:B7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-28 00:57 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="11" r:id="rId15"/>
-    <sheet name="Discontinued" sheetId="12" r:id="rId16"/>
-    <sheet name="Legit Codes" sheetId="13" r:id="rId17"/>
+    <sheet name="Alt Codes" sheetId="14" r:id="rId18"/>
+    <sheet name="Discontinued" sheetId="15" r:id="rId19"/>
+    <sheet name="Legit Codes" sheetId="16" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -48193,22 +48193,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">dominic-smith</t>
+          <t xml:space="preserve">airport-shannon</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARCHER MR200</t>
+          <t xml:space="preserve">GVCH1000MSR</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MR200</t>
+          <t xml:space="preserve">GVCH10000MSR</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">LTE/5G Gateway AC750 Wireless Dual Band 4G LTE Router</t>
+          <t xml:space="preserve">10000mAH Slim Magnetic Powerbank Charger - Magsafe compatiable - USB-C Charging - Magnetic wireless 5w/7.5w/10w/15w - LCD Power level disply</t>
         </is>
       </c>
     </row>
@@ -48220,17 +48220,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARCHERC50V3</t>
+          <t xml:space="preserve">ARCHER MR200</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARCHER C50V3</t>
+          <t xml:space="preserve">MR200</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wi-Fi 5 Router AC1200 Dual Band Wireless Cable Router</t>
+          <t xml:space="preserve">LTE/5G Gateway AC750 Wireless Dual Band 4G LTE Router</t>
         </is>
       </c>
     </row>
@@ -48242,17 +48242,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECOM4KIT</t>
+          <t xml:space="preserve">ARCHERC50V3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECOM4 KIT</t>
+          <t xml:space="preserve">ARCHER C50V3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+          <t xml:space="preserve">Wi-Fi 5 Router AC1200 Dual Band Wireless Cable Router</t>
         </is>
       </c>
     </row>
@@ -48264,17 +48264,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DVPSR760HB.CEK</t>
+          <t xml:space="preserve">DECOM4KIT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DVPSR760HBCEK</t>
+          <t xml:space="preserve">DECOM4 KIT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony DVD player with Picture enhcancing technology</t>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
         </is>
       </c>
     </row>
@@ -48286,17 +48286,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTSD40.CEK</t>
+          <t xml:space="preserve">DVPSR760HB.CEK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTSD40CEK</t>
+          <t xml:space="preserve">DVPSR760HBCEK</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony 2.1chl Soundbar with powerful Wireless Subwoofer inc</t>
+          <t xml:space="preserve">Sony DVD player with Picture enhcancing technology</t>
         </is>
       </c>
     </row>
@@ -48308,17 +48308,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTSF150.CEK</t>
+          <t xml:space="preserve">HTSD40.CEK</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTSF150CEK</t>
+          <t xml:space="preserve">HTSD40CEK</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony 2chl Single Soundbar with Bluetooth</t>
+          <t xml:space="preserve">Sony 2.1chl Soundbar with powerful Wireless Subwoofer inc</t>
         </is>
       </c>
     </row>
@@ -48330,17 +48330,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICF506.CEK</t>
+          <t xml:space="preserve">HTSF150.CEK</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICF506CEK</t>
+          <t xml:space="preserve">HTSF150CEK</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony portable AM/FM radio</t>
+          <t xml:space="preserve">Sony 2chl Single Soundbar with Bluetooth</t>
         </is>
       </c>
     </row>
@@ -48352,17 +48352,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFC1B.CEK</t>
+          <t xml:space="preserve">ICF506.CEK</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFC1BCEK</t>
+          <t xml:space="preserve">ICF506CEK</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Black AM/FM clock radio</t>
+          <t xml:space="preserve">Sony portable AM/FM radio</t>
         </is>
       </c>
     </row>
@@ -48374,17 +48374,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFC1W.CEK</t>
+          <t xml:space="preserve">ICFC1B.CEK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFC1WCEK</t>
+          <t xml:space="preserve">ICFC1BCEK</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony White AM/FM clock radio</t>
+          <t xml:space="preserve">Sony Black AM/FM clock radio</t>
         </is>
       </c>
     </row>
@@ -48396,17 +48396,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAXMINIFILM</t>
+          <t xml:space="preserve">ICFC1W.CEK</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAX MINI FILM</t>
+          <t xml:space="preserve">ICFC1WCEK</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+          <t xml:space="preserve">Sony White AM/FM clock radio</t>
         </is>
       </c>
     </row>
@@ -48418,17 +48418,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10B.CE7</t>
+          <t xml:space="preserve">INSTAXMINIFILM</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10BCE7</t>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Black Portable BT Speaker</t>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
         </is>
       </c>
     </row>
@@ -48440,17 +48440,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10W.CE7</t>
+          <t xml:space="preserve">SRSULT10B.CE7</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10WCE7</t>
+          <t xml:space="preserve">SRSULT10BCE7</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony White Portable BT Speaker</t>
+          <t xml:space="preserve">Sony Black Portable BT Speaker</t>
         </is>
       </c>
     </row>
@@ -48462,17 +48462,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100B.CE7</t>
+          <t xml:space="preserve">SRSULT10W.CE7</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100BCE7</t>
+          <t xml:space="preserve">SRSULT10WCE7</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Black Waterproof BT Speaker, EXTRA BASS</t>
+          <t xml:space="preserve">Sony White Portable BT Speaker</t>
         </is>
       </c>
     </row>
@@ -48484,17 +48484,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100D.CE7</t>
+          <t xml:space="preserve">SRSXB100B.CE7</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100DCE7</t>
+          <t xml:space="preserve">SRSXB100BCE7</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Orange Compact BT Wirelss Spkr</t>
+          <t xml:space="preserve">Sony Black Waterproof BT Speaker, EXTRA BASS</t>
         </is>
       </c>
     </row>
@@ -48506,17 +48506,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100H.CE7</t>
+          <t xml:space="preserve">SRSXB100D.CE7</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100HCE7</t>
+          <t xml:space="preserve">SRSXB100DCE7</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Light Grey Waterproof BT Speaker, EXTRA BASS</t>
+          <t xml:space="preserve">Sony Orange Compact BT Wirelss Spkr</t>
         </is>
       </c>
     </row>
@@ -48528,17 +48528,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100L.CE7</t>
+          <t xml:space="preserve">SRSXB100H.CE7</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100LCE7</t>
+          <t xml:space="preserve">SRSXB100HCE7</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Light Blue Waterproof BT Speaker, EXTRA BASS</t>
+          <t xml:space="preserve">Sony Light Grey Waterproof BT Speaker, EXTRA BASS</t>
         </is>
       </c>
     </row>
@@ -48550,17 +48550,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC100</t>
+          <t xml:space="preserve">SRSXB100L.CE7</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C100</t>
+          <t xml:space="preserve">SRSXB100LCE7</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+          <t xml:space="preserve">Sony Light Blue Waterproof BT Speaker, EXTRA BASS</t>
         </is>
       </c>
     </row>
@@ -48572,17 +48572,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC200</t>
+          <t xml:space="preserve">TAPOC100</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C200</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
@@ -48594,17 +48594,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC310</t>
+          <t xml:space="preserve">TAPOC200</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C310</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
@@ -48616,17 +48616,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510B</t>
+          <t xml:space="preserve">TAPOC310</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510B</t>
+          <t xml:space="preserve">TAPO C310</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
         </is>
       </c>
     </row>
@@ -48638,12 +48638,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">TAPOL510B</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">TAPO L510B</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -48660,17 +48660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530B</t>
+          <t xml:space="preserve">TAPOL510E</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530B</t>
+          <t xml:space="preserve">TAPO L510E</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
@@ -48682,12 +48682,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530E</t>
+          <t xml:space="preserve">TAPOL530B</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530E</t>
+          <t xml:space="preserve">TAPO L530B</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -48704,17 +48704,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL9205</t>
+          <t xml:space="preserve">TAPOL530E</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L9205</t>
+          <t xml:space="preserve">TAPO L530E</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -48726,17 +48726,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOP100</t>
+          <t xml:space="preserve">TAPOL9205</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO P100</t>
+          <t xml:space="preserve">TAPO L9205</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
         </is>
       </c>
     </row>
@@ -48748,17 +48748,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KITV2</t>
+          <t xml:space="preserve">TAPOP100</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KIT V2</t>
+          <t xml:space="preserve">TAPO P100</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
         </is>
       </c>
     </row>
@@ -48770,39 +48770,39 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t xml:space="preserve">WPA8631PKIT</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t xml:space="preserve">WPA8631P KIT</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link AV1300/AV2000 Powerline Adapter AV1300 Gigabit</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">joyces</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ARCHERAX55</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ARCHER AX55</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Wi-Fi 6 Router AX3000 Dual-Band Wi-Fi 6 Router</t>
         </is>
       </c>
     </row>
@@ -48814,17 +48814,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">DVR2SD32GBU3</t>
+          <t xml:space="preserve">ARCHERAX55</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+          <t xml:space="preserve">ARCHER AX55</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+          <t xml:space="preserve">TP-Link Wi-Fi 6 Router AX3000 Dual-Band Wi-Fi 6 Router</t>
         </is>
       </c>
     </row>
@@ -48836,17 +48836,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">DVR2SD64GBU3</t>
+          <t xml:space="preserve">DVR2SD32GBU3</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -48858,61 +48858,61 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
+          <t xml:space="preserve">DVR2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t xml:space="preserve">DVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t xml:space="preserve">rob-test</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t xml:space="preserve">WPA7517KITV2</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t xml:space="preserve">WPA7517KIT V2</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">soundstore</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GVPS110BLK</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GVPS110BK</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Groove  Black Portable CD Player</t>
         </is>
       </c>
     </row>
@@ -48924,17 +48924,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">GVPS110BLK</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">GVPS110BK</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">Groove  Black Portable CD Player</t>
         </is>
       </c>
     </row>
@@ -48946,22 +48946,44 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t xml:space="preserve">TAPOP100H</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOH100</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D36"/>
+  <autoFilter ref="A1:D37"/>
 </worksheet>
 </file>
 
@@ -49119,7 +49141,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVBT1200BK</t>
+          <t xml:space="preserve">112000</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -49131,7 +49153,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAS36WA</t>
+          <t xml:space="preserve">130055</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -49143,7 +49165,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1023R</t>
+          <t xml:space="preserve">DVPSR760HB</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -49155,7 +49177,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDRZX310APBCE7</t>
+          <t xml:space="preserve">GVBT1200BK</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -49167,7 +49189,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">MS816</t>
+          <t xml:space="preserve">HAS36WA</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -49176,7 +49198,43 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1023R</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX310APBCE7</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS816</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B10"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-28 00:58 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="14" r:id="rId18"/>
-    <sheet name="Discontinued" sheetId="15" r:id="rId19"/>
-    <sheet name="Legit Codes" sheetId="16" r:id="rId20"/>
+    <sheet name="Alt Codes" sheetId="17" r:id="rId21"/>
+    <sheet name="Discontinued" sheetId="18" r:id="rId22"/>
+    <sheet name="Legit Codes" sheetId="19" r:id="rId23"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -48897,93 +48897,511 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C501GW</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC501GW</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Pan/Tilt 4G LTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H100</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOH100</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L530B</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L530E</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L9205</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NB-NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-HDMI1010R</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1010R</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 1m, gold-plated connectors, 19-pin male-male, black</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-HDMI1030R</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1030R</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 3m, gold-plated connectors, 19-pin male-male, black</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-INSTAXMINI12P</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAXMINI12P</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instax Mini 12 Powder Pink camera No Film</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-INSTAXMINIFILM</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC100</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC200</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC410KIT</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC410KIT</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Security Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC500</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC500</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Outdoor Camera Tapo Pan/Tilt Security Wi-Fi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TP62VR</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP62VR</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 2m, white</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TP65VR</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP65VR</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 5m, white</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-AC750</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RE200</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Range Extender AC750 Dual Band Wi-Fi Universal</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t xml:space="preserve">rob-test</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t xml:space="preserve">WPA7517KITV2</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t xml:space="preserve">WPA7517KIT V2</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="54">
+      <c r="A54" t="inlineStr">
         <is>
           <t xml:space="preserve">soundstore</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t xml:space="preserve">GVPS110BLK</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t xml:space="preserve">GVPS110BK</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t xml:space="preserve">Groove  Black Portable CD Player</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t xml:space="preserve">soundstore</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOL510E</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPO L510E</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="56">
+      <c r="A56" t="inlineStr">
         <is>
           <t xml:space="preserve">soundstore</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOP100H</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOH100</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D37"/>
+  <autoFilter ref="A1:D56"/>
 </worksheet>
 </file>
 
@@ -49009,7 +49427,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">FB1001100EUS</t>
+          <t xml:space="preserve">DECOE42PK</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -49021,7 +49439,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFP27.CE7</t>
+          <t xml:space="preserve">FB1001100EUS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -49033,7 +49451,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFP37.CE7</t>
+          <t xml:space="preserve">ICFP27.CE7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -49045,7 +49463,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRS-NS7</t>
+          <t xml:space="preserve">ICFP37.CE7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -49057,7 +49475,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC2250100EUS</t>
+          <t xml:space="preserve">SRS-NS7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -49069,7 +49487,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4250P100EUS</t>
+          <t xml:space="preserve">VMC2250100EUS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -49081,7 +49499,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4260P100EUS</t>
+          <t xml:space="preserve">VMC4250P100EUS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -49093,7 +49511,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4360B100EUS</t>
+          <t xml:space="preserve">VMC4260P100EUS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -49102,8 +49520,20 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4360B100EUS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B10"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-28 01:59 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="17" r:id="rId21"/>
-    <sheet name="Discontinued" sheetId="18" r:id="rId22"/>
-    <sheet name="Legit Codes" sheetId="19" r:id="rId23"/>
+    <sheet name="Alt Codes" sheetId="20" r:id="rId24"/>
+    <sheet name="Discontinued" sheetId="21" r:id="rId25"/>
+    <sheet name="Legit Codes" sheetId="22" r:id="rId26"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -49400,8 +49400,206 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4KIT</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4 KIT</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC100</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC200</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO P100</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D56"/>
+  <autoFilter ref="A1:D65"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Catalog update — Mark Sutcliffe — 2026-08-28 08:17 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="20" r:id="rId24"/>
-    <sheet name="Discontinued" sheetId="21" r:id="rId25"/>
-    <sheet name="Legit Codes" sheetId="22" r:id="rId26"/>
+    <sheet name="Alt Codes" sheetId="23" r:id="rId27"/>
+    <sheet name="Discontinued" sheetId="24" r:id="rId28"/>
+    <sheet name="Legit Codes" sheetId="25" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -49757,7 +49757,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">100315</t>
+          <t xml:space="preserve">1000000409</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -49769,7 +49769,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">112000</t>
+          <t xml:space="preserve">112048</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -49781,7 +49781,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">130055</t>
+          <t xml:space="preserve">429776</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -49793,7 +49793,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">DVPSR760HB</t>
+          <t xml:space="preserve">430002</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -49805,7 +49805,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVBT1200BK</t>
+          <t xml:space="preserve">430009</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -49817,7 +49817,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAS36WA</t>
+          <t xml:space="preserve">661401</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -49829,7 +49829,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1023R</t>
+          <t xml:space="preserve">661406</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -49841,7 +49841,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDRZX310APBCE7</t>
+          <t xml:space="preserve">ARIVA160COMBO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -49853,7 +49853,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">MS816</t>
+          <t xml:space="preserve">ARIVA175COMBO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -49862,7 +49862,115 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GO528</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GO540</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GO554</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1023R</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB1S</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS816</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOA200</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOD235</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UB500</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B19"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Mark Sutcliffe — 2026-08-28 08:22 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="23" r:id="rId27"/>
-    <sheet name="Discontinued" sheetId="24" r:id="rId28"/>
-    <sheet name="Legit Codes" sheetId="25" r:id="rId29"/>
+    <sheet name="Alt Codes" sheetId="26" r:id="rId30"/>
+    <sheet name="Discontinued" sheetId="27" r:id="rId31"/>
+    <sheet name="Legit Codes" sheetId="28" r:id="rId32"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -48440,17 +48440,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10B.CE7</t>
+          <t xml:space="preserve">NBDVRS2SD128GBU NEXTBASE 128GB U3 MICROSD CARD AND MICRO</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10BCE7</t>
+          <t xml:space="preserve">NBDVRS2SD128GBU3</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Black Portable BT Speaker</t>
+          <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -48462,17 +48462,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10W.CE7</t>
+          <t xml:space="preserve">NBDVRS2SD32GBU3 NEXTBASE 32GB U3 MICROSD CARD AND MICROS</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10WCE7</t>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony White Portable BT Speaker</t>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -48484,17 +48484,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100B.CE7</t>
+          <t xml:space="preserve">NBDVRS2SD64GBU3 NEXTBASE 64GB U3 MICROSD CARD &amp; ADAPTER</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100BCE7</t>
+          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Black Waterproof BT Speaker, EXTRA BASS</t>
+          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -48506,17 +48506,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100D.CE7</t>
+          <t xml:space="preserve">SRSULT10B.CE7</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100DCE7</t>
+          <t xml:space="preserve">SRSULT10BCE7</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Orange Compact BT Wirelss Spkr</t>
+          <t xml:space="preserve">Sony Black Portable BT Speaker</t>
         </is>
       </c>
     </row>
@@ -48528,17 +48528,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100H.CE7</t>
+          <t xml:space="preserve">SRSULT10W.CE7</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100HCE7</t>
+          <t xml:space="preserve">SRSULT10WCE7</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Light Grey Waterproof BT Speaker, EXTRA BASS</t>
+          <t xml:space="preserve">Sony White Portable BT Speaker</t>
         </is>
       </c>
     </row>
@@ -48550,17 +48550,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100L.CE7</t>
+          <t xml:space="preserve">SRSXB100B.CE7</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100LCE7</t>
+          <t xml:space="preserve">SRSXB100BCE7</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Light Blue Waterproof BT Speaker, EXTRA BASS</t>
+          <t xml:space="preserve">Sony Black Waterproof BT Speaker, EXTRA BASS</t>
         </is>
       </c>
     </row>
@@ -48572,17 +48572,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC100</t>
+          <t xml:space="preserve">SRSXB100D.CE7</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C100</t>
+          <t xml:space="preserve">SRSXB100DCE7</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+          <t xml:space="preserve">Sony Orange Compact BT Wirelss Spkr</t>
         </is>
       </c>
     </row>
@@ -48594,17 +48594,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC200</t>
+          <t xml:space="preserve">SRSXB100H.CE7</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C200</t>
+          <t xml:space="preserve">SRSXB100HCE7</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+          <t xml:space="preserve">Sony Light Grey Waterproof BT Speaker, EXTRA BASS</t>
         </is>
       </c>
     </row>
@@ -48616,17 +48616,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC310</t>
+          <t xml:space="preserve">SRSXB100L.CE7</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C310</t>
+          <t xml:space="preserve">SRSXB100LCE7</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
+          <t xml:space="preserve">Sony Light Blue Waterproof BT Speaker, EXTRA BASS</t>
         </is>
       </c>
     </row>
@@ -48638,17 +48638,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510B</t>
+          <t xml:space="preserve">TAPOC100</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510B</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
@@ -48660,17 +48660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">TAPOC200</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
@@ -48682,17 +48682,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530B</t>
+          <t xml:space="preserve">TAPOC310</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530B</t>
+          <t xml:space="preserve">TAPO C310</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
         </is>
       </c>
     </row>
@@ -48704,17 +48704,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530E</t>
+          <t xml:space="preserve">TAPOL510B</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530E</t>
+          <t xml:space="preserve">TAPO L510B</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
@@ -48726,17 +48726,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL9205</t>
+          <t xml:space="preserve">TAPOL510E</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L9205</t>
+          <t xml:space="preserve">TAPO L510E</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
@@ -48748,17 +48748,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOP100</t>
+          <t xml:space="preserve">TAPOL530B</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO P100</t>
+          <t xml:space="preserve">TAPO L530B</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -48770,17 +48770,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KITV2</t>
+          <t xml:space="preserve">TAPOL530E</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KIT V2</t>
+          <t xml:space="preserve">TAPO L530E</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -48792,193 +48792,193 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO P100</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WFC710NBCE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WFC710NBCE7</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In ear buds</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t xml:space="preserve">WPA8631PKIT</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t xml:space="preserve">WPA8631P KIT</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link AV1300/AV2000 Powerline Adapter AV1300 Gigabit</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="34">
+      <c r="A34" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t xml:space="preserve">ARCHERAX55</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t xml:space="preserve">ARCHER AX55</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Wi-Fi 6 Router AX3000 Dual-Band Wi-Fi 6 Router</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t xml:space="preserve">DVR2SD32GBU3</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="36">
+      <c r="A36" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t xml:space="preserve">DVR2SD64GBU3</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD64GBU3</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t xml:space="preserve">DVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C501GW</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOC501GW</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Outdoor Camera Pan/Tilt 4G LTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">H100</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOH100</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L530B</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO L530B</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L530E</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO L530E</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -48990,17 +48990,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">L9205</t>
+          <t xml:space="preserve">C501GW</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L9205</t>
+          <t xml:space="preserve">TAPOC501GW</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Pan/Tilt 4G LTE</t>
         </is>
       </c>
     </row>
@@ -49012,17 +49012,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">NB-NBDVRS2SD32GBU3</t>
+          <t xml:space="preserve">H100</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+          <t xml:space="preserve">TAPOH100</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
         </is>
       </c>
     </row>
@@ -49034,17 +49034,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-HDMI1010R</t>
+          <t xml:space="preserve">L530B</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1010R</t>
+          <t xml:space="preserve">TAPO L530B</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 1m, gold-plated connectors, 19-pin male-male, black</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -49056,17 +49056,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-HDMI1030R</t>
+          <t xml:space="preserve">L530E</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1030R</t>
+          <t xml:space="preserve">TAPO L530E</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 3m, gold-plated connectors, 19-pin male-male, black</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -49078,17 +49078,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-INSTAXMINI12P</t>
+          <t xml:space="preserve">L9205</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAXMINI12P</t>
+          <t xml:space="preserve">TAPO L9205</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instax Mini 12 Powder Pink camera No Film</t>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
         </is>
       </c>
     </row>
@@ -49100,17 +49100,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-INSTAXMINIFILM</t>
+          <t xml:space="preserve">NB-NBDVRS2SD32GBU3</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAX MINI FILM</t>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -49122,17 +49122,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC100</t>
+          <t xml:space="preserve">PT-HDMI1010R</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C100</t>
+          <t xml:space="preserve">HDMI1010R</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 1m, gold-plated connectors, 19-pin male-male, black</t>
         </is>
       </c>
     </row>
@@ -49144,17 +49144,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC200</t>
+          <t xml:space="preserve">PT-HDMI1030R</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C200</t>
+          <t xml:space="preserve">HDMI1030R</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 3m, gold-plated connectors, 19-pin male-male, black</t>
         </is>
       </c>
     </row>
@@ -49166,17 +49166,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC410KIT</t>
+          <t xml:space="preserve">PT-INSTAXMINI12P</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC410KIT</t>
+          <t xml:space="preserve">INSTAXMINI12P</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Security Kit</t>
+          <t xml:space="preserve">Instax Mini 12 Powder Pink camera No Film</t>
         </is>
       </c>
     </row>
@@ -49188,17 +49188,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC500</t>
+          <t xml:space="preserve">PT-INSTAXMINIFILM</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC500</t>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Outdoor Camera Tapo Pan/Tilt Security Wi-Fi Camera</t>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
         </is>
       </c>
     </row>
@@ -49210,17 +49210,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TP62VR</t>
+          <t xml:space="preserve">PT-TAPOC100</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP62VR</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 2m, white</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
@@ -49232,17 +49232,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TP65VR</t>
+          <t xml:space="preserve">PT-TAPOC200</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP65VR</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 5m, white</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
@@ -49254,17 +49254,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510B</t>
+          <t xml:space="preserve">PT-TAPOC410KIT</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510B</t>
+          <t xml:space="preserve">TAPOC410KIT</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Security Kit</t>
         </is>
       </c>
     </row>
@@ -49276,17 +49276,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">PT-TAPOC500</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">TAPOC500</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">Smart Outdoor Camera Tapo Pan/Tilt Security Wi-Fi Camera</t>
         </is>
       </c>
     </row>
@@ -49298,68 +49298,68 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-AC750</t>
+          <t xml:space="preserve">PT-TP62VR</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">RE200</t>
+          <t xml:space="preserve">TP62VR</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wi-Fi 5 Range Extender AC750 Dual Band Wi-Fi Universal</t>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 2m, white</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">rob-test</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KITV2</t>
+          <t xml:space="preserve">PT-TP65VR</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KIT V2</t>
+          <t xml:space="preserve">TP65VR</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 5m, white</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">soundstore</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVPS110BLK</t>
+          <t xml:space="preserve">TAPOL510B</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVPS110BK</t>
+          <t xml:space="preserve">TAPO L510B</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Groove  Black Portable CD Player</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">soundstore</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -49381,110 +49381,110 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-AC750</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RE200</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Range Extender AC750 Dual Band Wi-Fi Universal</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rob-test</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t xml:space="preserve">soundstore</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BLK</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BK</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groove  Black Portable CD Player</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOP100H</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOH100</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D60" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tj-omahony</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DECOM4KIT</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DECOM4 KIT</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tj-omahony</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOC100</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO C100</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tj-omahony</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOC200</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO C200</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tj-omahony</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOL510B</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO L510B</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
@@ -49496,17 +49496,17 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">DECOM4KIT</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">DECOM4 KIT</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
         </is>
       </c>
     </row>
@@ -49518,17 +49518,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530B</t>
+          <t xml:space="preserve">TAPOC100</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530B</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
@@ -49540,17 +49540,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530E</t>
+          <t xml:space="preserve">TAPOC200</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530E</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
@@ -49562,17 +49562,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL9205</t>
+          <t xml:space="preserve">TAPOL510B</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L9205</t>
+          <t xml:space="preserve">TAPO L510B</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
@@ -49584,22 +49584,110 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
           <t xml:space="preserve">TAPOP100</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C69" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPO P100</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D69" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D65"/>
+  <autoFilter ref="A1:D69"/>
 </worksheet>
 </file>
 
@@ -49769,7 +49857,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">112048</t>
+          <t xml:space="preserve">112000</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -49781,7 +49869,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">429776</t>
+          <t xml:space="preserve">112048</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -49793,7 +49881,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">430002</t>
+          <t xml:space="preserve">130055</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -49805,7 +49893,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">430009</t>
+          <t xml:space="preserve">429776</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -49817,7 +49905,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">661401</t>
+          <t xml:space="preserve">430002</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -49829,7 +49917,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">661406</t>
+          <t xml:space="preserve">430009</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -49841,7 +49929,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARIVA160COMBO</t>
+          <t xml:space="preserve">661401</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -49853,7 +49941,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARIVA175COMBO</t>
+          <t xml:space="preserve">661406</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -49865,7 +49953,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">GO528</t>
+          <t xml:space="preserve">ARIVA160COMBO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -49877,7 +49965,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GO540</t>
+          <t xml:space="preserve">ARIVA175COMBO</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -49889,7 +49977,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">GO554</t>
+          <t xml:space="preserve">GO528</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -49901,7 +49989,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1023R</t>
+          <t xml:space="preserve">GO540</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -49913,7 +50001,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">KB1S</t>
+          <t xml:space="preserve">GO554</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -49925,7 +50013,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">MS816</t>
+          <t xml:space="preserve">HDMI1023R</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -49937,7 +50025,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOA200</t>
+          <t xml:space="preserve">KB1S</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -49949,7 +50037,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOD235</t>
+          <t xml:space="preserve">MS816</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -49961,7 +50049,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">UB500</t>
+          <t xml:space="preserve">TAPOA200</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -49970,7 +50058,31 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOD235</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UB500</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B19"/>
+  <autoFilter ref="A1:B21"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-28 09:45 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="26" r:id="rId30"/>
-    <sheet name="Discontinued" sheetId="27" r:id="rId31"/>
-    <sheet name="Legit Codes" sheetId="28" r:id="rId32"/>
+    <sheet name="Alt Codes" sheetId="29" r:id="rId33"/>
+    <sheet name="Discontinued" sheetId="30" r:id="rId34"/>
+    <sheet name="Legit Codes" sheetId="31" r:id="rId35"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -49845,7 +49845,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1000000409</t>
+          <t xml:space="preserve">100315</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -49869,7 +49869,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">112048</t>
+          <t xml:space="preserve">130055</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -49881,7 +49881,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">130055</t>
+          <t xml:space="preserve">421725</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -49893,7 +49893,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">429776</t>
+          <t xml:space="preserve">421726</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -49905,7 +49905,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">430002</t>
+          <t xml:space="preserve">421766</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -49917,7 +49917,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">430009</t>
+          <t xml:space="preserve">429905</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -49929,7 +49929,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">661401</t>
+          <t xml:space="preserve">429910</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -49941,7 +49941,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">661406</t>
+          <t xml:space="preserve">429911</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -49953,7 +49953,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARIVA160COMBO</t>
+          <t xml:space="preserve">DVPSR760HB</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -49965,7 +49965,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARIVA175COMBO</t>
+          <t xml:space="preserve">GVBT1200BK</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -49977,7 +49977,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">GO528</t>
+          <t xml:space="preserve">HAFR9UCWU</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -49989,7 +49989,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GO540</t>
+          <t xml:space="preserve">HAS36WA</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -50001,7 +50001,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">GO554</t>
+          <t xml:space="preserve">HDMI1023R</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -50013,7 +50013,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1023R</t>
+          <t xml:space="preserve">MDRZX310APBCE7</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -50025,7 +50025,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">KB1S</t>
+          <t xml:space="preserve">MS816</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -50034,55 +50034,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MS816</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Confirmed valid — add to catalog</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOA200</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Confirmed valid — add to catalog</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOD235</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Confirmed valid — add to catalog</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UB500</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Confirmed valid — add to catalog</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B21"/>
+  <autoFilter ref="A1:B17"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-28 10:08 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="29" r:id="rId33"/>
-    <sheet name="Discontinued" sheetId="30" r:id="rId34"/>
-    <sheet name="Legit Codes" sheetId="31" r:id="rId35"/>
+    <sheet name="Alt Codes" sheetId="32" r:id="rId36"/>
+    <sheet name="Discontinued" sheetId="33" r:id="rId37"/>
+    <sheet name="Legit Codes" sheetId="34" r:id="rId38"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -48193,110 +48193,110 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPBAE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APBCE7</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPLIAE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APLICE7</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Blue In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPPIAE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APPICE7</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Pink In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPWAE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APWCE7</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t xml:space="preserve">airport-shannon</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t xml:space="preserve">GVCH1000MSR</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t xml:space="preserve">GVCH10000MSR</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t xml:space="preserve">10000mAH Slim Magnetic Powerbank Charger - Magsafe compatiable - USB-C Charging - Magnetic wireless 5w/7.5w/10w/15w - LCD Power level disply</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dominic-smith</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ARCHER MR200</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MR200</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LTE/5G Gateway AC750 Wireless Dual Band 4G LTE Router</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dominic-smith</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ARCHERC50V3</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ARCHER C50V3</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wi-Fi 5 Router AC1200 Dual Band Wireless Cable Router</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dominic-smith</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DECOM4KIT</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DECOM4 KIT</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">dominic-smith</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DVPSR760HB.CEK</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DVPSR760HBCEK</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sony DVD player with Picture enhcancing technology</t>
         </is>
       </c>
     </row>
@@ -48308,17 +48308,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTSD40.CEK</t>
+          <t xml:space="preserve">ARCHER MR200</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTSD40CEK</t>
+          <t xml:space="preserve">MR200</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony 2.1chl Soundbar with powerful Wireless Subwoofer inc</t>
+          <t xml:space="preserve">LTE/5G Gateway AC750 Wireless Dual Band 4G LTE Router</t>
         </is>
       </c>
     </row>
@@ -48330,17 +48330,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTSF150.CEK</t>
+          <t xml:space="preserve">ARCHERC50V3</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HTSF150CEK</t>
+          <t xml:space="preserve">ARCHER C50V3</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony 2chl Single Soundbar with Bluetooth</t>
+          <t xml:space="preserve">Wi-Fi 5 Router AC1200 Dual Band Wireless Cable Router</t>
         </is>
       </c>
     </row>
@@ -48352,17 +48352,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICF506.CEK</t>
+          <t xml:space="preserve">DECOM4KIT</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICF506CEK</t>
+          <t xml:space="preserve">DECOM4 KIT</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony portable AM/FM radio</t>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
         </is>
       </c>
     </row>
@@ -48374,17 +48374,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFC1B.CEK</t>
+          <t xml:space="preserve">DVPSR760HB.CEK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFC1BCEK</t>
+          <t xml:space="preserve">DVPSR760HBCEK</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Black AM/FM clock radio</t>
+          <t xml:space="preserve">Sony DVD player with Picture enhcancing technology</t>
         </is>
       </c>
     </row>
@@ -48396,17 +48396,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFC1W.CEK</t>
+          <t xml:space="preserve">HTSD40.CEK</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFC1WCEK</t>
+          <t xml:space="preserve">HTSD40CEK</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony White AM/FM clock radio</t>
+          <t xml:space="preserve">Sony 2.1chl Soundbar with powerful Wireless Subwoofer inc</t>
         </is>
       </c>
     </row>
@@ -48418,17 +48418,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAXMINIFILM</t>
+          <t xml:space="preserve">HTSF150.CEK</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAX MINI FILM</t>
+          <t xml:space="preserve">HTSF150CEK</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+          <t xml:space="preserve">Sony 2chl Single Soundbar with Bluetooth</t>
         </is>
       </c>
     </row>
@@ -48440,17 +48440,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD128GBU NEXTBASE 128GB U3 MICROSD CARD AND MICRO</t>
+          <t xml:space="preserve">ICF506.CEK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD128GBU3</t>
+          <t xml:space="preserve">ICF506CEK</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
+          <t xml:space="preserve">Sony portable AM/FM radio</t>
         </is>
       </c>
     </row>
@@ -48462,17 +48462,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD32GBU3 NEXTBASE 32GB U3 MICROSD CARD AND MICROS</t>
+          <t xml:space="preserve">ICFC1B.CEK</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+          <t xml:space="preserve">ICFC1BCEK</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+          <t xml:space="preserve">Sony Black AM/FM clock radio</t>
         </is>
       </c>
     </row>
@@ -48484,17 +48484,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD64GBU3 NEXTBASE 64GB U3 MICROSD CARD &amp; ADAPTER</t>
+          <t xml:space="preserve">ICFC1W.CEK</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
+          <t xml:space="preserve">ICFC1WCEK</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
+          <t xml:space="preserve">Sony White AM/FM clock radio</t>
         </is>
       </c>
     </row>
@@ -48506,17 +48506,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10B.CE7</t>
+          <t xml:space="preserve">INSTAXMINIFILM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10BCE7</t>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Black Portable BT Speaker</t>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
         </is>
       </c>
     </row>
@@ -48528,17 +48528,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10W.CE7</t>
+          <t xml:space="preserve">NBDVRS2SD128GBU NEXTBASE 128GB U3 MICROSD CARD AND MICRO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSULT10WCE7</t>
+          <t xml:space="preserve">NBDVRS2SD128GBU3</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony White Portable BT Speaker</t>
+          <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -48550,17 +48550,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100B.CE7</t>
+          <t xml:space="preserve">NBDVRS2SD32GBU3 NEXTBASE 32GB U3 MICROSD CARD AND MICROS</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100BCE7</t>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Black Waterproof BT Speaker, EXTRA BASS</t>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -48572,17 +48572,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100D.CE7</t>
+          <t xml:space="preserve">NBDVRS2SD64GBU3 NEXTBASE 64GB U3 MICROSD CARD &amp; ADAPTER</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100DCE7</t>
+          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Orange Compact BT Wirelss Spkr</t>
+          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -48594,17 +48594,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100H.CE7</t>
+          <t xml:space="preserve">SRSULT10B.CE7</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100HCE7</t>
+          <t xml:space="preserve">SRSULT10BCE7</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Light Grey Waterproof BT Speaker, EXTRA BASS</t>
+          <t xml:space="preserve">Sony Black Portable BT Speaker</t>
         </is>
       </c>
     </row>
@@ -48616,17 +48616,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100L.CE7</t>
+          <t xml:space="preserve">SRSULT10W.CE7</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRSXB100LCE7</t>
+          <t xml:space="preserve">SRSULT10WCE7</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Light Blue Waterproof BT Speaker, EXTRA BASS</t>
+          <t xml:space="preserve">Sony White Portable BT Speaker</t>
         </is>
       </c>
     </row>
@@ -48638,17 +48638,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC100</t>
+          <t xml:space="preserve">SRSXB100B.CE7</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C100</t>
+          <t xml:space="preserve">SRSXB100BCE7</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+          <t xml:space="preserve">Sony Black Waterproof BT Speaker, EXTRA BASS</t>
         </is>
       </c>
     </row>
@@ -48660,17 +48660,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC200</t>
+          <t xml:space="preserve">SRSXB100D.CE7</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C200</t>
+          <t xml:space="preserve">SRSXB100DCE7</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+          <t xml:space="preserve">Sony Orange Compact BT Wirelss Spkr</t>
         </is>
       </c>
     </row>
@@ -48682,17 +48682,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC310</t>
+          <t xml:space="preserve">SRSXB100H.CE7</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C310</t>
+          <t xml:space="preserve">SRSXB100HCE7</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
+          <t xml:space="preserve">Sony Light Grey Waterproof BT Speaker, EXTRA BASS</t>
         </is>
       </c>
     </row>
@@ -48704,17 +48704,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510B</t>
+          <t xml:space="preserve">SRSXB100L.CE7</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510B</t>
+          <t xml:space="preserve">SRSXB100LCE7</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">Sony Light Blue Waterproof BT Speaker, EXTRA BASS</t>
         </is>
       </c>
     </row>
@@ -48726,17 +48726,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">TAPOC100</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
@@ -48748,17 +48748,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530B</t>
+          <t xml:space="preserve">TAPOC200</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530B</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
@@ -48770,17 +48770,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530E</t>
+          <t xml:space="preserve">TAPOC310</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530E</t>
+          <t xml:space="preserve">TAPO C310</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
         </is>
       </c>
     </row>
@@ -48792,17 +48792,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL9205</t>
+          <t xml:space="preserve">TAPOL510B</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L9205</t>
+          <t xml:space="preserve">TAPO L510B</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
@@ -48814,17 +48814,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOP100</t>
+          <t xml:space="preserve">TAPOL510E</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO P100</t>
+          <t xml:space="preserve">TAPO L510E</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
@@ -48836,17 +48836,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">WFC710NBCE</t>
+          <t xml:space="preserve">TAPOL530B</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t xml:space="preserve">WFC710NBCE7</t>
+          <t xml:space="preserve">TAPO L530B</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sony Black In ear buds</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -48858,17 +48858,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KITV2</t>
+          <t xml:space="preserve">TAPOL530E</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KIT V2</t>
+          <t xml:space="preserve">TAPO L530E</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -48880,193 +48880,193 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO P100</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WFC710NBCE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WFC710NBCE7</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In ear buds</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t xml:space="preserve">WPA8631PKIT</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t xml:space="preserve">WPA8631P KIT</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link AV1300/AV2000 Powerline Adapter AV1300 Gigabit</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="38">
+      <c r="A38" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t xml:space="preserve">ARCHERAX55</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t xml:space="preserve">ARCHER AX55</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Wi-Fi 6 Router AX3000 Dual-Band Wi-Fi 6 Router</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="39">
+      <c r="A39" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t xml:space="preserve">DVR2SD32GBU3</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t xml:space="preserve">DVR2SD64GBU3</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD64GBU3</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t xml:space="preserve">DVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C501GW</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOC501GW</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Outdoor Camera Pan/Tilt 4G LTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">H100</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOH100</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L530B</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO L530B</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L530E</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO L530E</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -49078,17 +49078,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">L9205</t>
+          <t xml:space="preserve">C501GW</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L9205</t>
+          <t xml:space="preserve">TAPOC501GW</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Pan/Tilt 4G LTE</t>
         </is>
       </c>
     </row>
@@ -49100,17 +49100,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">NB-NBDVRS2SD32GBU3</t>
+          <t xml:space="preserve">H100</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+          <t xml:space="preserve">TAPOH100</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
         </is>
       </c>
     </row>
@@ -49122,17 +49122,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-HDMI1010R</t>
+          <t xml:space="preserve">L530B</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1010R</t>
+          <t xml:space="preserve">TAPO L530B</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 1m, gold-plated connectors, 19-pin male-male, black</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -49144,17 +49144,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-HDMI1030R</t>
+          <t xml:space="preserve">L530E</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1030R</t>
+          <t xml:space="preserve">TAPO L530E</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 3m, gold-plated connectors, 19-pin male-male, black</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -49166,17 +49166,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-INSTAXMINI12P</t>
+          <t xml:space="preserve">L9205</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAXMINI12P</t>
+          <t xml:space="preserve">TAPO L9205</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instax Mini 12 Powder Pink camera No Film</t>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
         </is>
       </c>
     </row>
@@ -49188,17 +49188,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-INSTAXMINIFILM</t>
+          <t xml:space="preserve">NB-NBDVRS2SD32GBU3</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAX MINI FILM</t>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -49210,17 +49210,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC100</t>
+          <t xml:space="preserve">PT-HDMI1010R</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C100</t>
+          <t xml:space="preserve">HDMI1010R</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 1m, gold-plated connectors, 19-pin male-male, black</t>
         </is>
       </c>
     </row>
@@ -49232,17 +49232,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC200</t>
+          <t xml:space="preserve">PT-HDMI1030R</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C200</t>
+          <t xml:space="preserve">HDMI1030R</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 3m, gold-plated connectors, 19-pin male-male, black</t>
         </is>
       </c>
     </row>
@@ -49254,17 +49254,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC410KIT</t>
+          <t xml:space="preserve">PT-INSTAXMINI12P</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC410KIT</t>
+          <t xml:space="preserve">INSTAXMINI12P</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Security Kit</t>
+          <t xml:space="preserve">Instax Mini 12 Powder Pink camera No Film</t>
         </is>
       </c>
     </row>
@@ -49276,17 +49276,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC500</t>
+          <t xml:space="preserve">PT-INSTAXMINIFILM</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC500</t>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Outdoor Camera Tapo Pan/Tilt Security Wi-Fi Camera</t>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
         </is>
       </c>
     </row>
@@ -49298,17 +49298,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TP62VR</t>
+          <t xml:space="preserve">PT-TAPOC100</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP62VR</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 2m, white</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
@@ -49320,17 +49320,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TP65VR</t>
+          <t xml:space="preserve">PT-TAPOC200</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP65VR</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 5m, white</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
@@ -49342,17 +49342,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510B</t>
+          <t xml:space="preserve">PT-TAPOC410KIT</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510B</t>
+          <t xml:space="preserve">TAPOC410KIT</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Security Kit</t>
         </is>
       </c>
     </row>
@@ -49364,17 +49364,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">PT-TAPOC500</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">TAPOC500</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">Smart Outdoor Camera Tapo Pan/Tilt Security Wi-Fi Camera</t>
         </is>
       </c>
     </row>
@@ -49386,68 +49386,68 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-AC750</t>
+          <t xml:space="preserve">PT-TP62VR</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">RE200</t>
+          <t xml:space="preserve">TP62VR</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wi-Fi 5 Range Extender AC750 Dual Band Wi-Fi Universal</t>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 2m, white</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">rob-test</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KITV2</t>
+          <t xml:space="preserve">PT-TP65VR</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KIT V2</t>
+          <t xml:space="preserve">TP65VR</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 5m, white</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">soundstore</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVPS110BLK</t>
+          <t xml:space="preserve">TAPOL510B</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVPS110BK</t>
+          <t xml:space="preserve">TAPO L510B</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Groove  Black Portable CD Player</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">soundstore</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -49469,110 +49469,110 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-AC750</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RE200</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Range Extender AC750 Dual Band Wi-Fi Universal</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rob-test</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t xml:space="preserve">soundstore</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BLK</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BK</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groove  Black Portable CD Player</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOP100H</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOH100</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D64" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tj-omahony</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DECOM4KIT</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DECOM4 KIT</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tj-omahony</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOC100</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO C100</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tj-omahony</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOC200</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO C200</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tj-omahony</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOL510B</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO L510B</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
@@ -49584,17 +49584,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">DECOM4KIT</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">DECOM4 KIT</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
         </is>
       </c>
     </row>
@@ -49606,17 +49606,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530B</t>
+          <t xml:space="preserve">TAPOC100</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530B</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
@@ -49628,17 +49628,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530E</t>
+          <t xml:space="preserve">TAPOC200</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530E</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
@@ -49650,17 +49650,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL9205</t>
+          <t xml:space="preserve">TAPOL510B</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L9205</t>
+          <t xml:space="preserve">TAPO L510B</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
@@ -49672,22 +49672,110 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t xml:space="preserve">TAPOP100</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPO P100</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D73" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D69"/>
+  <autoFilter ref="A1:D73"/>
 </worksheet>
 </file>
 
@@ -49713,7 +49801,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECOE42PK</t>
+          <t xml:space="preserve">1000000409</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -49725,7 +49813,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">FB1001100EUS</t>
+          <t xml:space="preserve">DECOE42PK</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -49737,7 +49825,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFP27.CE7</t>
+          <t xml:space="preserve">FB1001100EUS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -49749,7 +49837,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFP37.CE7</t>
+          <t xml:space="preserve">ICFP27.CE7</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -49761,7 +49849,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRS-NS7</t>
+          <t xml:space="preserve">ICFP37.CE7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -49773,7 +49861,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC2250100EUS</t>
+          <t xml:space="preserve">SRS-NS7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -49785,7 +49873,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4250P100EUS</t>
+          <t xml:space="preserve">VMC2250100EUS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -49797,7 +49885,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4260P100EUS</t>
+          <t xml:space="preserve">VMC4250P100EUS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -49809,7 +49897,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4360B100EUS</t>
+          <t xml:space="preserve">VMC4260P100EUS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -49818,8 +49906,20 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4360B100EUS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B10"/>
+  <autoFilter ref="A1:B11"/>
 </worksheet>
 </file>
 
@@ -49869,7 +49969,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">130055</t>
+          <t xml:space="preserve">112048</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -49881,7 +49981,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">421725</t>
+          <t xml:space="preserve">130055</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -49893,7 +49993,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">421726</t>
+          <t xml:space="preserve">421725</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -49905,7 +50005,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">421766</t>
+          <t xml:space="preserve">421726</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -49917,7 +50017,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">429905</t>
+          <t xml:space="preserve">421766</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -49929,7 +50029,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">429910</t>
+          <t xml:space="preserve">429776</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -49941,7 +50041,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">429911</t>
+          <t xml:space="preserve">429905</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -49953,7 +50053,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">DVPSR760HB</t>
+          <t xml:space="preserve">429910</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -49965,7 +50065,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVBT1200BK</t>
+          <t xml:space="preserve">429911</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -49977,7 +50077,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAFR9UCWU</t>
+          <t xml:space="preserve">430002</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -49989,7 +50089,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAS36WA</t>
+          <t xml:space="preserve">430009</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -50001,7 +50101,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1023R</t>
+          <t xml:space="preserve">661401</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -50013,7 +50113,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDRZX310APBCE7</t>
+          <t xml:space="preserve">661406</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -50025,7 +50125,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">MS816</t>
+          <t xml:space="preserve">ARIVA160COMBO</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -50034,7 +50134,187 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARIVA175COMBO</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVPSR760HB</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GO528</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GO540</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GO554</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVBT1200BK</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HAFR9UCWU</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HAS36WA</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1023R</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">KB1S</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX310APBCE7</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS816</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOA200</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOD235</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UB500</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B17"/>
+  <autoFilter ref="A1:B32"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-28 18:19 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="32" r:id="rId36"/>
-    <sheet name="Discontinued" sheetId="33" r:id="rId37"/>
-    <sheet name="Legit Codes" sheetId="34" r:id="rId38"/>
+    <sheet name="Alt Codes" sheetId="35" r:id="rId39"/>
+    <sheet name="Discontinued" sheetId="36" r:id="rId40"/>
+    <sheet name="Legit Codes" sheetId="37" r:id="rId41"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-29 10:02 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="35" r:id="rId39"/>
-    <sheet name="Discontinued" sheetId="36" r:id="rId40"/>
-    <sheet name="Legit Codes" sheetId="37" r:id="rId41"/>
+    <sheet name="Alt Codes" sheetId="38" r:id="rId42"/>
+    <sheet name="Discontinued" sheetId="39" r:id="rId43"/>
+    <sheet name="Legit Codes" sheetId="40" r:id="rId44"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -50041,7 +50041,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">429905</t>
+          <t xml:space="preserve">429832</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -50053,7 +50053,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">429910</t>
+          <t xml:space="preserve">429905</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -50065,7 +50065,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">429911</t>
+          <t xml:space="preserve">429910</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -50077,7 +50077,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">430002</t>
+          <t xml:space="preserve">429911</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -50089,7 +50089,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">430009</t>
+          <t xml:space="preserve">430002</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -50101,7 +50101,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">661401</t>
+          <t xml:space="preserve">430009</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -50113,7 +50113,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">661406</t>
+          <t xml:space="preserve">661401</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -50125,7 +50125,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARIVA160COMBO</t>
+          <t xml:space="preserve">661406</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -50137,7 +50137,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">ARIVA175COMBO</t>
+          <t xml:space="preserve">ARIVA160COMBO</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -50149,7 +50149,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">DVPSR760HB</t>
+          <t xml:space="preserve">ARIVA175COMBO</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -50161,7 +50161,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">GO528</t>
+          <t xml:space="preserve">DVPSR760HB</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -50173,7 +50173,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">GO540</t>
+          <t xml:space="preserve">GO528</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -50185,7 +50185,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">GO554</t>
+          <t xml:space="preserve">GO540</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -50197,7 +50197,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVBT1200BK</t>
+          <t xml:space="preserve">GO554</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -50209,7 +50209,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAFR9UCWU</t>
+          <t xml:space="preserve">GVBT1200BK</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -50221,7 +50221,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">HAS36WA</t>
+          <t xml:space="preserve">HAFR9UCWU</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -50233,7 +50233,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1023R</t>
+          <t xml:space="preserve">HAS36WA</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -50245,7 +50245,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">KB1S</t>
+          <t xml:space="preserve">HDMI1023R</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -50257,7 +50257,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDRZX310APBCE7</t>
+          <t xml:space="preserve">KB1S</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -50269,7 +50269,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">MS816</t>
+          <t xml:space="preserve">MDRZX310APBCE7</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -50281,7 +50281,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOA200</t>
+          <t xml:space="preserve">MS816</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -50293,7 +50293,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOD235</t>
+          <t xml:space="preserve">TAPOA200</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -50305,7 +50305,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">UB500</t>
+          <t xml:space="preserve">TAPOD235</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -50314,7 +50314,19 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UB500</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B32"/>
+  <autoFilter ref="A1:B33"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-29 18:00 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="38" r:id="rId42"/>
-    <sheet name="Discontinued" sheetId="39" r:id="rId43"/>
-    <sheet name="Legit Codes" sheetId="40" r:id="rId44"/>
+    <sheet name="Alt Codes" sheetId="41" r:id="rId45"/>
+    <sheet name="Discontinued" sheetId="42" r:id="rId46"/>
+    <sheet name="Legit Codes" sheetId="43" r:id="rId47"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -48985,198 +48985,198 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH5000MS</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH5000MSR</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5000mAH Slim Magnetic Powerbank Charger - USB-C input - USB-A output x 2 - USB-C output x 1 - USB-A to USB-C charging cable inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPB</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APBCE7</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPL</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APLICE7</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Blue In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPW</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APWCE7</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX110BA</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX110BAE</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Black Supra-aural closed-ear Headphones with a 12Hz–22kHz</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t xml:space="preserve">ARCHERAX55</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t xml:space="preserve">ARCHER AX55</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Wi-Fi 6 Router AX3000 Dual-Band Wi-Fi 6 Router</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t xml:space="preserve">DVR2SD32GBU3</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="45">
+      <c r="A45" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t xml:space="preserve">DVR2SD64GBU3</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD64GBU3</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t xml:space="preserve">joyces</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B46" t="inlineStr">
         <is>
           <t xml:space="preserve">DVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C46" t="inlineStr">
         <is>
           <t xml:space="preserve">NBDVRS2SD128GBU3</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">C501GW</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOC501GW</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Outdoor Camera Pan/Tilt 4G LTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">H100</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPOH100</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L530B</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO L530B</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L530E</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO L530E</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king-moffatt</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">L9205</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAPO L9205</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
         </is>
       </c>
     </row>
@@ -49188,17 +49188,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">NB-NBDVRS2SD32GBU3</t>
+          <t xml:space="preserve">C501GW</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+          <t xml:space="preserve">TAPOC501GW</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Pan/Tilt 4G LTE</t>
         </is>
       </c>
     </row>
@@ -49210,17 +49210,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-HDMI1010R</t>
+          <t xml:space="preserve">H100</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1010R</t>
+          <t xml:space="preserve">TAPOH100</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 1m, gold-plated connectors, 19-pin male-male, black</t>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
         </is>
       </c>
     </row>
@@ -49232,17 +49232,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-HDMI1030R</t>
+          <t xml:space="preserve">L530B</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI1030R</t>
+          <t xml:space="preserve">TAPO L530B</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 3m, gold-plated connectors, 19-pin male-male, black</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -49254,17 +49254,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-INSTAXMINI12P</t>
+          <t xml:space="preserve">L530E</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAXMINI12P</t>
+          <t xml:space="preserve">TAPO L530E</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instax Mini 12 Powder Pink camera No Film</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
         </is>
       </c>
     </row>
@@ -49276,17 +49276,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-INSTAXMINIFILM</t>
+          <t xml:space="preserve">L9205</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t xml:space="preserve">INSTAX MINI FILM</t>
+          <t xml:space="preserve">TAPO L9205</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
         </is>
       </c>
     </row>
@@ -49298,17 +49298,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC100</t>
+          <t xml:space="preserve">NB-NBDVRS2SD32GBU3</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C100</t>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
         </is>
       </c>
     </row>
@@ -49320,17 +49320,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC200</t>
+          <t xml:space="preserve">PT-HDMI1010R</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C200</t>
+          <t xml:space="preserve">HDMI1010R</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 1m, gold-plated connectors, 19-pin male-male, black</t>
         </is>
       </c>
     </row>
@@ -49342,17 +49342,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC410KIT</t>
+          <t xml:space="preserve">PT-HDMI1030R</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC410KIT</t>
+          <t xml:space="preserve">HDMI1030R</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Security Kit</t>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 3m, gold-plated connectors, 19-pin male-male, black</t>
         </is>
       </c>
     </row>
@@ -49364,17 +49364,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TAPOC500</t>
+          <t xml:space="preserve">PT-INSTAXMINI12P</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC500</t>
+          <t xml:space="preserve">INSTAXMINI12P</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Outdoor Camera Tapo Pan/Tilt Security Wi-Fi Camera</t>
+          <t xml:space="preserve">Instax Mini 12 Powder Pink camera No Film</t>
         </is>
       </c>
     </row>
@@ -49386,17 +49386,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TP62VR</t>
+          <t xml:space="preserve">PT-INSTAXMINIFILM</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP62VR</t>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 2m, white</t>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
         </is>
       </c>
     </row>
@@ -49408,17 +49408,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">PT-TP65VR</t>
+          <t xml:space="preserve">PT-TAPOC100</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP65VR</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 5m, white</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
@@ -49430,17 +49430,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510B</t>
+          <t xml:space="preserve">PT-TAPOC200</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510B</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
@@ -49452,17 +49452,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">PT-TAPOC410KIT</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">TAPOC410KIT</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Security Kit</t>
         </is>
       </c>
     </row>
@@ -49474,78 +49474,78 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-AC750</t>
+          <t xml:space="preserve">PT-TAPOC500</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">RE200</t>
+          <t xml:space="preserve">TAPOC500</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wi-Fi 5 Range Extender AC750 Dual Band Wi-Fi Universal</t>
+          <t xml:space="preserve">Smart Outdoor Camera Tapo Pan/Tilt Security Wi-Fi Camera</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">rob-test</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KITV2</t>
+          <t xml:space="preserve">PT-TP62VR</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">WPA7517KIT V2</t>
+          <t xml:space="preserve">TP62VR</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 2m, white</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">soundstore</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVPS110BLK</t>
+          <t xml:space="preserve">PT-TP65VR</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVPS110BK</t>
+          <t xml:space="preserve">TP65VR</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Groove  Black Portable CD Player</t>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 5m, white</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">soundstore</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">TAPOL510B</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">TAPO L510B</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -49557,105 +49557,105 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">soundstore</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOP100H</t>
+          <t xml:space="preserve">TAPOL510E</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOH100</t>
+          <t xml:space="preserve">TAPO L510E</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">king-moffatt</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECOM4KIT</t>
+          <t xml:space="preserve">TP-AC750</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECOM4 KIT</t>
+          <t xml:space="preserve">RE200</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+          <t xml:space="preserve">Wi-Fi 5 Range Extender AC750 Dual Band Wi-Fi Universal</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">rob-test</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC100</t>
+          <t xml:space="preserve">WPA7517KITV2</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C100</t>
+          <t xml:space="preserve">WPA7517KIT V2</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">soundstore</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC200</t>
+          <t xml:space="preserve">GVPS110BLK</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C200</t>
+          <t xml:space="preserve">GVPS110BK</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+          <t xml:space="preserve">Groove  Black Portable CD Player</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">soundstore</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510B</t>
+          <t xml:space="preserve">TAPOL510E</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510B</t>
+          <t xml:space="preserve">TAPO L510E</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -49667,22 +49667,22 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">soundstore</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">TAPOP100H</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">TAPOH100</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
         </is>
       </c>
     </row>
@@ -49694,17 +49694,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530B</t>
+          <t xml:space="preserve">DECOM4KIT</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530B</t>
+          <t xml:space="preserve">DECOM4 KIT</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
         </is>
       </c>
     </row>
@@ -49716,17 +49716,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530E</t>
+          <t xml:space="preserve">TAPOC100</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530E</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
@@ -49738,17 +49738,17 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL9205</t>
+          <t xml:space="preserve">TAPOC200</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L9205</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
@@ -49760,22 +49760,132 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t xml:space="preserve">TAPOP100</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
+      <c r="C78" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPO P100</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D78" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D73"/>
+  <autoFilter ref="A1:D78"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-30 13:24 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Alt Codes" sheetId="41" r:id="rId45"/>
     <sheet name="Discontinued" sheetId="42" r:id="rId46"/>
     <sheet name="Legit Codes" sheetId="43" r:id="rId47"/>
+    <sheet name="Excluded Codes" sheetId="44" r:id="rId48"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>
@@ -50439,4 +50440,96 @@
   </sheetData>
   <autoFilter ref="A1:B33"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Retailer</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>BDPS1700B.CEK</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>BDPS3700B.CEK</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BDPS5500B.CEK</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MS763</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-30 22:15 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,10 +9,10 @@
   </bookViews>
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Alt Codes" sheetId="41" r:id="rId45"/>
-    <sheet name="Discontinued" sheetId="42" r:id="rId46"/>
-    <sheet name="Legit Codes" sheetId="43" r:id="rId47"/>
     <sheet name="Excluded Codes" sheetId="44" r:id="rId48"/>
+    <sheet name="Alt Codes" sheetId="45" r:id="rId49"/>
+    <sheet name="Discontinued" sheetId="46" r:id="rId50"/>
+    <sheet name="Legit Codes" sheetId="47" r:id="rId51"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-30 22:29 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -10,9 +10,9 @@
   <sheets>
     <sheet name="Product Catalog" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Excluded Codes" sheetId="44" r:id="rId48"/>
-    <sheet name="Alt Codes" sheetId="45" r:id="rId49"/>
-    <sheet name="Discontinued" sheetId="46" r:id="rId50"/>
-    <sheet name="Legit Codes" sheetId="47" r:id="rId51"/>
+    <sheet name="Alt Codes" sheetId="48" r:id="rId52"/>
+    <sheet name="Discontinued" sheetId="49" r:id="rId53"/>
+    <sheet name="Legit Codes" sheetId="50" r:id="rId54"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Alt Codes'!$A$1:$D$9</definedName>

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-30 22:35 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -1,26 +1,5 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="5" state="visible" r:id="rId5"/>
-  </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$K$1021</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Alt Codes'!$A$1:$D$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Discontinued'!$A$1:$B$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Legit Codes'!$A$1:$B$33</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
-</workbook>
+<file path=xl/workbook.xml><workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"><workbookPr/><workbookProtection/><bookViews><workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/></bookViews><sheets><sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/><sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="2" state="visible" r:id="rId2"/><sheet name="Alt Codes" sheetId="6" r:id="rId8"/><sheet name="Discontinued" sheetId="7" r:id="rId9"/><sheet name="Legit Codes" sheetId="8" r:id="rId10"/></sheets><definedNames><definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$K$1021</definedName><definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Alt Codes'!$A$1:$D$78</definedName><definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Discontinued'!$A$1:$B$11</definedName><definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Legit Codes'!$A$1:$B$33</definedName></definedNames><calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/></workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -51932,4 +51911,1913 @@
   <autoFilter ref="A1:B33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="42" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer Code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peats Code</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPBAE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APBCE7</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPLIAE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APLICE7</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Blue In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPPIAE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APPICE7</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Pink In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPWAE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APWCE7</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-shannon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH1000MSR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH10000MSR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10000mAH Slim Magnetic Powerbank Charger - Magsafe compatiable - USB-C Charging - Magnetic wireless 5w/7.5w/10w/15w - LCD Power level disply</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHER MR200</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MR200</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LTE/5G Gateway AC750 Wireless Dual Band 4G LTE Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHERC50V3</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHER C50V3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Router AC1200 Dual Band Wireless Cable Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4KIT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4 KIT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVPSR760HB.CEK</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVPSR760HBCEK</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony DVD player with Picture enhcancing technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSD40.CEK</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSD40CEK</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony 2.1chl Soundbar with powerful Wireless Subwoofer inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSF150.CEK</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSF150CEK</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony 2chl Single Soundbar with Bluetooth</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICF506.CEK</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICF506CEK</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony portable AM/FM radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1B.CEK</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1BCEK</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black AM/FM clock radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1W.CEK</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1WCEK</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White AM/FM clock radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAXMINIFILM</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD128GBU NEXTBASE 128GB U3 MICROSD CARD AND MICRO</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD128GBU3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3 NEXTBASE 32GB U3 MICROSD CARD AND MICROS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD64GBU3 NEXTBASE 64GB U3 MICROSD CARD &amp; ADAPTER</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10B.CE7</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10BCE7</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black Portable BT Speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10W.CE7</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10WCE7</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White Portable BT Speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100B.CE7</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100BCE7</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black Waterproof BT Speaker, EXTRA BASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100D.CE7</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100DCE7</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Orange Compact BT Wirelss Spkr</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100H.CE7</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100HCE7</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Light Grey Waterproof BT Speaker, EXTRA BASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100L.CE7</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100LCE7</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Light Blue Waterproof BT Speaker, EXTRA BASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC100</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC200</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC310</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C310</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO P100</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WFC710NBCE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WFC710NBCE7</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In ear buds</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA8631PKIT</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA8631P KIT</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link AV1300/AV2000 Powerline Adapter AV1300 Gigabit</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH5000MS</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH5000MSR</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5000mAH Slim Magnetic Powerbank Charger - USB-C input - USB-A output x 2 - USB-C output x 1 - USB-A to USB-C charging cable inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPB</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APBCE7</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPL</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APLICE7</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Blue In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPW</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APWCE7</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX110BA</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX110BAE</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Black Supra-aural closed-ear Headphones with a 12Hz–22kHz</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHERAX55</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHER AX55</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Wi-Fi 6 Router AX3000 Dual-Band Wi-Fi 6 Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVR2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVR2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVRS2SD128GBU3</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD128GBU3</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C501GW</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC501GW</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Pan/Tilt 4G LTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H100</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOH100</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L530B</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L530E</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L9205</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NB-NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-HDMI1010R</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1010R</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 1m, gold-plated connectors, 19-pin male-male, black</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-HDMI1030R</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1030R</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 3m, gold-plated connectors, 19-pin male-male, black</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-INSTAXMINI12P</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAXMINI12P</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instax Mini 12 Powder Pink camera No Film</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-INSTAXMINIFILM</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC100</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC200</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC410KIT</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC410KIT</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Security Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC500</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC500</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Outdoor Camera Tapo Pan/Tilt Security Wi-Fi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TP62VR</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP62VR</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 2m, white</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TP65VR</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP65VR</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 5m, white</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-AC750</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RE200</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Range Extender AC750 Dual Band Wi-Fi Universal</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rob-test</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BLK</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BK</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groove  Black Portable CD Player</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100H</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOH100</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4KIT</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4 KIT</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC100</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC200</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO P100</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D78"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1000000409</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOE42PK</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FB1001100EUS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFP27.CE7</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFP37.CE7</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRS-NS7</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC2250100EUS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4250P100EUS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4260P100EUS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4360B100EUS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B11"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="44" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS816</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-30 22:51 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="6" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="7" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="8" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$K$1021</definedName>
@@ -51932,4 +51932,1913 @@
   <autoFilter ref="A1:B33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="42" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer Code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Peats Code</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPBAE</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APBCE7</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPLIAE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APLICE7</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Blue In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPPIAE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APPICE7</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Pink In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-cork</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPWAE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APWCE7</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">airport-shannon</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH1000MSR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH10000MSR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10000mAH Slim Magnetic Powerbank Charger - Magsafe compatiable - USB-C Charging - Magnetic wireless 5w/7.5w/10w/15w - LCD Power level disply</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHER MR200</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MR200</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LTE/5G Gateway AC750 Wireless Dual Band 4G LTE Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHERC50V3</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHER C50V3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Router AC1200 Dual Band Wireless Cable Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4KIT</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4 KIT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVPSR760HB.CEK</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVPSR760HBCEK</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony DVD player with Picture enhcancing technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSD40.CEK</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSD40CEK</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony 2.1chl Soundbar with powerful Wireless Subwoofer inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSF150.CEK</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HTSF150CEK</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony 2chl Single Soundbar with Bluetooth</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICF506.CEK</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICF506CEK</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony portable AM/FM radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1B.CEK</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1BCEK</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black AM/FM clock radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1W.CEK</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFC1WCEK</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White AM/FM clock radio</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAXMINIFILM</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD128GBU NEXTBASE 128GB U3 MICROSD CARD AND MICRO</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD128GBU3</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3 NEXTBASE 32GB U3 MICROSD CARD AND MICROS</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD64GBU3 NEXTBASE 64GB U3 MICROSD CARD &amp; ADAPTER</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10B.CE7</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10BCE7</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black Portable BT Speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10W.CE7</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSULT10WCE7</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White Portable BT Speaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100B.CE7</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100BCE7</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black Waterproof BT Speaker, EXTRA BASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100D.CE7</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100DCE7</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Orange Compact BT Wirelss Spkr</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100H.CE7</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100HCE7</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Light Grey Waterproof BT Speaker, EXTRA BASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100L.CE7</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRSXB100LCE7</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Light Blue Waterproof BT Speaker, EXTRA BASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC100</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC200</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC310</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C310</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO P100</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WFC710NBCE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WFC710NBCE7</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In ear buds</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dominic-smith</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA8631PKIT</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA8631P KIT</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link AV1300/AV2000 Powerline Adapter AV1300 Gigabit</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH5000MS</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVCH5000MSR</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5000mAH Slim Magnetic Powerbank Charger - USB-C input - USB-A output x 2 - USB-C output x 1 - USB-A to USB-C charging cable inc</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPB</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APBCE7</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Black In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPL</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APLICE7</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony Blue In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15LPW</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDREX15APWCE7</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sony White In Ear Smartphone earphone with silicon earbuds</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">easons</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX110BA</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX110BAE</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Black Supra-aural closed-ear Headphones with a 12Hz–22kHz</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHERAX55</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ARCHER AX55</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Wi-Fi 6 Router AX3000 Dual-Band Wi-Fi 6 Router</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVR2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVR2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD64GBU3</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 64GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">joyces</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DVRS2SD128GBU3</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD128GBU3</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 128GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C501GW</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC501GW</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Pan/Tilt 4G LTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">H100</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOH100</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L530B</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L530E</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">L9205</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NB-NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NBDVRS2SD32GBU3</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nextbase 32GB U3 microSD Card</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-HDMI1010R</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1010R</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 1m, gold-plated connectors, 19-pin male-male, black</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-HDMI1030R</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI1030R</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HDMI cable, Premium High Speed HDMI with Ethernet, 4K, UltraHD, 3m, gold-plated connectors, 19-pin male-male, black</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-INSTAXMINI12P</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAXMINI12P</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instax Mini 12 Powder Pink camera No Film</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-INSTAXMINIFILM</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC100</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC200</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC410KIT</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC410KIT</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Security Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TAPOC500</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC500</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Outdoor Camera Tapo Pan/Tilt Security Wi-Fi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TP62VR</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP62VR</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 2m, white</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PT-TP65VR</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP65VR</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ú/UTP Cat6 patch cable, LSZH, 5m, white</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king-moffatt</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-AC750</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RE200</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Range Extender AC750 Dual Band Wi-Fi Universal</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">rob-test</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BLK</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVPS110BK</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groove  Black Portable CD Player</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">soundstore</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100H</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOH100</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Sensor IoT Hub with Chime</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4KIT</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4 KIT</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC100</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC200</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOP100</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO P100</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D78"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="48" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1000000409</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOE42PK</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FB1001100EUS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFP27.CE7</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ICFP37.CE7</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SRS-NS7</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC2250100EUS</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4250P100EUS</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4260P100EUS</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4360B100EUS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B11"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="44" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Code</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MS816</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-30 23:50 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="6" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="7" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="8" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="9" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$K$1021</definedName>
@@ -53841,4 +53841,402 @@
   </sheetData>
   <autoFilter ref="A1:B2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Retailer</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>HTCT180.CEK</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>HTCT370.CEK</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HTG700.CEK</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>HTNT3.CEK</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>HTNT5.CEK</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HTS2000</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>HTS20R</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>HTS40R.CEK</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>HTSD35</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HTSD40.CEK</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HTSF150.CEK</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HTX8500</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>HTXF9000.CEK</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>HTXT100.CEK</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>HTZF9.CEK</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ICFP27.CE7</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ICFP37.CE7</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SA-RS3S.CEK</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SA-SW3.CEK</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SA-SW5.CEK</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SASW3.CEK</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SRS-NS7</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-30 23:52 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -53871,7 +53871,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>HTCT180.CEK</t>
+          <t>BDPS1700B.CEK</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -53888,7 +53888,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HTCT370.CEK</t>
+          <t>BDPS3700B.CEK</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -53905,7 +53905,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HTG700.CEK</t>
+          <t>BDPS5500B.CEK</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -53922,7 +53922,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HTNT3.CEK</t>
+          <t>DVPSR760HB.CEK</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -53939,7 +53939,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>HTNT5.CEK</t>
+          <t>HTA3000.CEK</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -53956,7 +53956,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HTS2000</t>
+          <t>HTA5000.CEK</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -53973,7 +53973,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HTS20R</t>
+          <t>HTA8000.CEK</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -53990,7 +53990,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>HTS40R.CEK</t>
+          <t>HTA9.CEK</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -54007,7 +54007,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HTSD35</t>
+          <t>HTA9000.CEK</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -54024,7 +54024,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HTSD40.CEK</t>
+          <t>HTA9M2.CEK</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -54041,7 +54041,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HTSF150.CEK</t>
+          <t>HTB600</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -54058,7 +54058,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>HTX8500</t>
+          <t>HTCT180.CEK</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -54075,7 +54075,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>HTXF9000.CEK</t>
+          <t>HTCT370.CEK</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -54092,7 +54092,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HTXT100.CEK</t>
+          <t>HTG700.CEK</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -54109,7 +54109,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HTZF9.CEK</t>
+          <t>HTNT3.CEK</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -54126,7 +54126,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ICFP27.CE7</t>
+          <t>HTNT5.CEK</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -54143,7 +54143,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ICFP37.CE7</t>
+          <t>HTS2000</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -54160,7 +54160,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SA-RS3S.CEK</t>
+          <t>HTS20R</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -54177,7 +54177,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SA-SW3.CEK</t>
+          <t>HTS40R.CEK</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -54194,7 +54194,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SA-SW5.CEK</t>
+          <t>HTSD35</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -54211,7 +54211,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SASW3.CEK</t>
+          <t>HTSD40.CEK</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -54228,10 +54228,775 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>HTSF150.CEK</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HTX8500</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HTXF9000.CEK</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>HTXT100.CEK</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HTZF9.CEK</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ICFP27.CE7</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ICFP37.CE7</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>MHCV02</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MHCV11.CEK</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>RRS-00007</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>SA-RS3S.CEK</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>SA-SW3.CEK</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>SA-SW5.CEK</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>SASW3.CEK</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>SRS-NS7</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SRSULT30H.CE7</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>SRSULT30W.CE7</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>SRSULT50B.CE7</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>SRSULT50W.CE7</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>SRSULT70B.EU8</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>SRSX77B.EU8</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>SRSXB100B.CE7</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>SRSXB100D.CE7</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>SRSXB100H.CE7</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>SRSXB100L.CE7</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>SRSXB10L.CE7</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>SRSXB10Y.CE7</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SRSXB13B.CE7</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SRSXB13L.CE7</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SRSXB13LI.CE7</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SRSXB21L.CE7</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>SRSXB23B.CE7</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>SRSXB23L.CE7</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>SRSXB23R.CE7</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>SRSXB30L.EU8</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>SRSXB33B.CE7</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>SRSXB33L.CE7</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>SRSXB33R.CE7</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>SRSXE200B.CE7</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>SRSXE200D.CE7</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>SRSXE200L.CE7</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>SRSXG300B.EU8</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>SRSXG300H.EU8</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SRSXG500B.EU8</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SRSXP500B.CEL</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>dominic-smith</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SRSXV500</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
         <is>
           <t>2026-08-30</t>
         </is>

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-30 23:54 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -8,10 +8,10 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="6" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="7" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="8" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="9" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="10" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="11" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="12" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$K$1021</definedName>
@@ -53745,7 +53745,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRS-NS7</t>
+          <t xml:space="preserve">KB1S</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -53757,7 +53757,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC2250100EUS</t>
+          <t xml:space="preserve">SRS-NS7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -53769,7 +53769,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4250P100EUS</t>
+          <t xml:space="preserve">VMC2250100EUS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -53781,7 +53781,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4260P100EUS</t>
+          <t xml:space="preserve">VMC4250P100EUS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -53793,17 +53793,29 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t xml:space="preserve">VMC4260P100EUS</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t xml:space="preserve">VMC4360B100EUS</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B12"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-31 06:24 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="9" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="10" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="11" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="12" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="13" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="14" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="15" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$K$1021</definedName>
@@ -53769,7 +53769,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC2250100EUS</t>
+          <t xml:space="preserve">TB114UK</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -53781,7 +53781,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4250P100EUS</t>
+          <t xml:space="preserve">TPM203TG</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -53793,7 +53793,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4260P100EUS</t>
+          <t xml:space="preserve">VMC2250100EUS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -53805,17 +53805,41 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t xml:space="preserve">VMC4250P100EUS</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">VMC4260P100EUS</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t xml:space="preserve">VMC4360B100EUS</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B12"/>
+  <autoFilter ref="A1:B14"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-31 06:41 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="9" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="13" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="14" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="15" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="16" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="17" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="18" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$K$1021</definedName>
@@ -53721,7 +53721,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFP27.CE7</t>
+          <t xml:space="preserve">HAS36WA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -53733,7 +53733,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICFP37.CE7</t>
+          <t xml:space="preserve">ICFP27.CE7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -53745,7 +53745,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">KB1S</t>
+          <t xml:space="preserve">ICFP37.CE7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -53757,7 +53757,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">SRS-NS7</t>
+          <t xml:space="preserve">KB1S</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -53769,7 +53769,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">TB114UK</t>
+          <t xml:space="preserve">SRS-NS7</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -53781,7 +53781,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">TPM203TG</t>
+          <t xml:space="preserve">TB114UK</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -53793,7 +53793,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC2250100EUS</t>
+          <t xml:space="preserve">TPM203TG</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -53805,7 +53805,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4250P100EUS</t>
+          <t xml:space="preserve">VMC2250100EUS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -53817,7 +53817,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">VMC4260P100EUS</t>
+          <t xml:space="preserve">VMC4250P100EUS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -53829,17 +53829,29 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t xml:space="preserve">VMC4260P100EUS</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t xml:space="preserve">VMC4360B100EUS</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B15"/>
 </worksheet>
 </file>
 
@@ -53865,17 +53877,53 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t xml:space="preserve">100315</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVBT1200BK</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX310APBCE7</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t xml:space="preserve">MS816</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed valid — add to catalog</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B2"/>
+  <autoFilter ref="A1:B5"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-31 09:28 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="9" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="16" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="17" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="18" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="19" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="20" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="21" r:id="rId23"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$K$1021</definedName>
@@ -576,8 +576,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProductCatalog" displayName="ProductCatalog" ref="A1:K1021" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:K1021"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProductCatalog" displayName="ProductCatalog" ref="A1:K1028" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:K1028"/>
   <tableColumns count="11">
     <tableColumn id="1" name="Brand"/>
     <tableColumn id="2" name="Peats Code"/>
@@ -775,7 +775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K1027"/>
+  <dimension ref="A1:K1028"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="29" min="1" max="1"/>
@@ -49562,8 +49562,37 @@
       <c r="J1027" t="inlineStr"/>
       <c r="K1027" t="inlineStr"/>
     </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr"/>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t xml:space="preserve">112004</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t xml:space="preserve">112004PEATS</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COAX PLUG TO PLUG 4M WHT</t>
+        </is>
+      </c>
+      <c r="E1028" t="inlineStr"/>
+      <c r="F1028" t="inlineStr"/>
+      <c r="G1028" t="inlineStr"/>
+      <c r="H1028" t="inlineStr"/>
+      <c r="I1028" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COAX PLUG TO PLUG 4M WHT</t>
+        </is>
+      </c>
+      <c r="J1028" t="inlineStr"/>
+      <c r="K1028" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K1021"/>
+  <autoFilter ref="A1:K1028"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -53463,203 +53492,511 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">stakelums</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECOM4KIT</t>
+          <t xml:space="preserve">112004PEATS</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">DECOM4 KIT</t>
+          <t xml:space="preserve">112004</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">stakelums</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC100</t>
+          <t xml:space="preserve">INSTAXMINIFILM</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C100</t>
+          <t xml:space="preserve">INSTAX MINI FILM</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+          <t xml:space="preserve">Instax Mini Film (Twin Pack)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">stakelums</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOC200</t>
+          <t xml:space="preserve">TAPO C610 KIT</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO C200</t>
+          <t xml:space="preserve">TAPOC610KIT</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Pan/Tilt Security Kit</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">stakelums</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510B</t>
+          <t xml:space="preserve">TAPO C615G KIT</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510B</t>
+          <t xml:space="preserve">TAPOC615GKIT</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">Battery Camera Solar-Powered Pan/Tilt 4G LTE Security</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">stakelums</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL510E</t>
+          <t xml:space="preserve">TAPO C660 KIT</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L510E</t>
+          <t xml:space="preserve">TAPOC660KIT</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+          <t xml:space="preserve">TP-Link Battery Camera Solar-Powered Pan/Tilt Security Kit</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">stakelums</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530B</t>
+          <t xml:space="preserve">TAPOC100</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530B</t>
+          <t xml:space="preserve">TAPO C100</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">stakelums</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL530E</t>
+          <t xml:space="preserve">TAPOC200</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L530E</t>
+          <t xml:space="preserve">TAPO C200</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">tj-omahony</t>
+          <t xml:space="preserve">stakelums</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPOL9205</t>
+          <t xml:space="preserve">TAPOC310</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPO L9205</t>
+          <t xml:space="preserve">TAPO C310</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+          <t xml:space="preserve">TP-Link Smart Outdoor Camera Security Wi-Fi</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
+          <t xml:space="preserve">stakelums</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stakelums</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stakelums</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stakelums</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stakelums</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">stakelums</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KITV2</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WPA7517KIT V2</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">AV600/AV1000 Powerline Adapter AV1000 Gigabit ac Wi-Fi Kit</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
           <t xml:space="preserve">tj-omahony</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
+      <c r="B84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4KIT</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECOM4 KIT</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wi-Fi 5 Mesh System AC1200 Whole-Home Wi-Fi System(3-pack)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC100</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C100</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Indoor Camera Home Security WiFi</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOC200</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO C200</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Smart Indoor Camera Pan/Tilt Home Security WiFi Camera</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510B</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510B</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL510E</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L510E</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Dimmable Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530B</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530B</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL530E</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L530E</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Bulb Wi-Fi Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPOL9205</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAPO L9205</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TP-Link Smart Strip Light</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tj-omahony</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPOP100</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t xml:space="preserve">TAPO P100</t>
         </is>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t xml:space="preserve">TP-Link Smart Plug Mini Wi-Fi Socket</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D78"/>
+  <autoFilter ref="A1:D92"/>
 </worksheet>
 </file>
 
@@ -53889,7 +54226,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVBT1200BK</t>
+          <t xml:space="preserve">112004</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -53901,7 +54238,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDRZX310APBCE7</t>
+          <t xml:space="preserve">GVBT1200BK</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -53913,17 +54250,29 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t xml:space="preserve">MDRZX310APBCE7</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t xml:space="preserve">MS816</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed valid — add to catalog</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B5"/>
+  <autoFilter ref="A1:B6"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Catalog update — Rob — 2026-08-31 14:49 UTC
</commit_message>
<xml_diff>
--- a/product_catalog.xlsx
+++ b/product_catalog.xlsx
@@ -9,9 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Product Catalog" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded Codes" sheetId="9" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="19" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="20" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="21" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alt Codes" sheetId="22" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discontinued" sheetId="23" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legit Codes" sheetId="24" r:id="rId26"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Catalog'!$A$1:$K$1021</definedName>
@@ -53507,7 +53507,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">COAX PLUG TO PLUG 4M WHT</t>
         </is>
       </c>
     </row>
@@ -54238,7 +54238,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">GVBT1200BK</t>
+          <t xml:space="preserve">421725</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -54250,7 +54250,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">MDRZX310APBCE7</t>
+          <t xml:space="preserve">421726</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -54262,17 +54262,101 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t xml:space="preserve">421766</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">429905</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">429910</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">429911</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GVBT1200BK</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HAFR9UCWU</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MDRZX310APBCE7</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirmed valid — add to catalog</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t xml:space="preserve">MS816</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t xml:space="preserve">Confirmed valid — add to catalog</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B6"/>
+  <autoFilter ref="A1:B13"/>
 </worksheet>
 </file>
 

</xml_diff>